<commit_message>
Publish revised Charles Bannerman Belt lineage
</commit_message>
<xml_diff>
--- a/LSC_Update_System.xlsx
+++ b/LSC_Update_System.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="R818fd2b95add4f1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="2" r:id="Ree2260e949d049b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rf6a39b1ad36c4fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Updates" sheetId="4" r:id="Rc3825060b1204ec5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="R6676fbec0a274fb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Export" sheetId="6" r:id="R19e4e37c7e4d4f63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="Re19d673467a445ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline" sheetId="2" r:id="R5440c47544f5463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rafeb7296dc2d47ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Updates" sheetId="4" r:id="Rfd4434d03244424c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="R708fda16524c41f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Export" sheetId="6" r:id="Ra5ffc5103f1748a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -824,11 +824,11 @@
       <x:c r="F2">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G2">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="H2">
-        <x:v>270</x:v>
+      <x:c r="G2" t="n">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="H2" t="n">
+        <x:v>404</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1290,11 +1290,11 @@
       </x:c>
       <x:c r="O2" s="6" t="n">
         <x:f>IF(B2="","",IF(K2="INVALID — CHECK RESULT TYPE","",VLOOKUP(B2,Baseline!$A$2:$H$10,7,FALSE)+IF(K2="Transfer",1,0)))</x:f>
-        <x:v>172</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="P2" s="6" t="n">
         <x:f>IF(B2="","",IF(K2="INVALID — CHECK RESULT TYPE","",VLOOKUP(B2,Baseline!$A$2:$H$10,8,FALSE)+IF(K2="Defence",1,0)))</x:f>
-        <x:v>270</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="Q2" s="5"/>
       <x:c r="R2" s="32" t="n">
@@ -5025,11 +5025,11 @@
       </x:c>
       <x:c r="E2" t="n">
         <x:f>IFERROR(LOOKUP(2,1/(Updates!$B$2:$B$100=A2),Updates!$O$2:$O$100),VLOOKUP(A2,Baseline!$A$2:$H$10,7,FALSE))</x:f>
-        <x:v>172</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="F2" t="n">
         <x:f>IFERROR(LOOKUP(2,1/(Updates!$B$2:$B$100=A2),Updates!$P$2:$P$100),VLOOKUP(A2,Baseline!$A$2:$H$10,8,FALSE))</x:f>
-        <x:v>270</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="G2" s="4" t="n">
         <x:f>IFERROR(LOOKUP(2,1/((Updates!$B$2:$B$100=A2)*(Updates!$F$2:$F$100&lt;&gt;"Completed")*(Updates!$F$2:$F$100&lt;&gt;"Cancelled")*(Updates!$F$2:$F$100&lt;&gt;"Postponed")),Updates!$C$2:$C$100),"TBD")</x:f>
@@ -5362,11 +5362,11 @@
       </x:c>
       <x:c r="E2" t="n">
         <x:f>Dashboard!E2</x:f>
-        <x:v>172</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="F2" t="n">
         <x:f>Dashboard!F2</x:f>
-        <x:v>270</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="G2" s="9" t="n">
         <x:f>Dashboard!G2</x:f>

</xml_diff>